<commit_message>
Round 2: live defaults, strike-first terms, Run Simulation flow, Primary shell and tables
- Remove saved-day defaults, saved input sets and the products API; defaults load live
- Strikes drive spreads, target, protection and floor; Option Type feeds every column
- Expiries on the underlying weekday nearest valuation plus months x 30.5 days
- Tenor rate curve anchored at valuation so Lower Maturity always resolves
- Bid or Offer as a surface parameter; per-leg and Day 1 volatility overrides
- Run Simulation with result gate, stale banner and edge-case popups with fixes
- Primary pill tabs, market strip, headline tables, Logic Atlas console
- Invariant tests, verification scripts and docs 01 to 10

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/samples/Hedging_Sheet_Vol_Surface_Sample.xlsx
+++ b/public/samples/Hedging_Sheet_Vol_Surface_Sample.xlsx
@@ -14,9 +14,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="37">
   <si>
-    <t>Volatility Surface Input · August 2026</t>
+    <t>Volatility Surface Input · October 2026</t>
   </si>
   <si>
     <t>Implied volatility in percent points by strike and expiry. Strike rows are live formulas of the reference prices times the Strike Change.</t>
@@ -40,7 +40,7 @@
     <t>Expiry Date</t>
   </si>
   <si>
-    <t>Surface Parameters · August 2026</t>
+    <t>Surface Parameters · October 2026</t>
   </si>
   <si>
     <t>Reference prices are the 100 percent anchors of the Strike Change columns. The Pricing Params table is read by expiry date.</t>
@@ -55,7 +55,7 @@
     <t>Month</t>
   </si>
   <si>
-    <t>August 2026</t>
+    <t>October 2026</t>
   </si>
   <si>
     <t>Reference Nifty Price</t>
@@ -74,6 +74,12 @@
   </si>
   <si>
     <t>Dividend Bid Offer Multiplier</t>
+  </si>
+  <si>
+    <t>Bid or Offer</t>
+  </si>
+  <si>
+    <t>Bid</t>
   </si>
   <si>
     <t>Date</t>
@@ -97,10 +103,19 @@
     <t>Rate Curve</t>
   </si>
   <si>
-    <t>Discount curve points in percent per annum. Leave the last points at the Premium Growth Rate to match the workbook.</t>
+    <t>Tenors in years from the valuation date, with rates in percent per annum. Linked points follow the Premium Growth Rate.</t>
+  </si>
+  <si>
+    <t>Tenor In Years</t>
   </si>
   <si>
     <t>Rate In Percent</t>
+  </si>
+  <si>
+    <t>Linked To Premium Growth Rate</t>
+  </si>
+  <si>
+    <t>Yes</t>
   </si>
   <si>
     <t>Implied Dividends</t>
@@ -2474,7 +2489,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H142"/>
+  <dimension ref="A1:H143"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
@@ -2623,49 +2638,37 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="6" t="s">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B17" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="C19" s="6" t="s">
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="D19" s="6" t="s">
+      <c r="B20" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="E19" s="6" t="s">
+      <c r="C20" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="F19" s="6" t="s">
+      <c r="D20" s="6" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="12">
-        <v>43916</v>
-      </c>
-      <c r="B20" s="15">
-        <v>0</v>
-      </c>
-      <c r="C20" s="15">
-        <v>0.0050000000000000044</v>
-      </c>
-      <c r="D20" s="15">
-        <v>0.065</v>
-      </c>
-      <c r="E20" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F20" s="15">
-        <v>0</v>
+      <c r="E20" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="12">
-        <v>44007</v>
+        <v>43916</v>
       </c>
       <c r="B21" s="15">
         <v>0</v>
@@ -2685,7 +2688,7 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="12">
-        <v>44042</v>
+        <v>44007</v>
       </c>
       <c r="B22" s="15">
         <v>0</v>
@@ -2705,7 +2708,7 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="12">
-        <v>44070</v>
+        <v>44042</v>
       </c>
       <c r="B23" s="15">
         <v>0</v>
@@ -2720,12 +2723,12 @@
         <v>0.03</v>
       </c>
       <c r="F23" s="15">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="12">
-        <v>44098</v>
+        <v>44070</v>
       </c>
       <c r="B24" s="15">
         <v>0</v>
@@ -2745,7 +2748,7 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="12">
-        <v>44133</v>
+        <v>44098</v>
       </c>
       <c r="B25" s="15">
         <v>0</v>
@@ -2760,12 +2763,12 @@
         <v>0.03</v>
       </c>
       <c r="F25" s="15">
-        <v>0.006</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="12">
-        <v>44160</v>
+        <v>44133</v>
       </c>
       <c r="B26" s="15">
         <v>0</v>
@@ -2785,7 +2788,7 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="12">
-        <v>44196</v>
+        <v>44160</v>
       </c>
       <c r="B27" s="15">
         <v>0</v>
@@ -2800,12 +2803,12 @@
         <v>0.03</v>
       </c>
       <c r="F27" s="15">
-        <v>0.0085</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="12">
-        <v>44224</v>
+        <v>44196</v>
       </c>
       <c r="B28" s="15">
         <v>0</v>
@@ -2825,7 +2828,7 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="12">
-        <v>44252</v>
+        <v>44224</v>
       </c>
       <c r="B29" s="15">
         <v>0</v>
@@ -2845,7 +2848,7 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="12">
-        <v>44280</v>
+        <v>44252</v>
       </c>
       <c r="B30" s="15">
         <v>0</v>
@@ -2860,21 +2863,21 @@
         <v>0.03</v>
       </c>
       <c r="F30" s="15">
-        <v>0.031</v>
+        <v>0.0085</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="12">
-        <v>44315</v>
+        <v>44280</v>
       </c>
       <c r="B31" s="15">
         <v>0</v>
       </c>
       <c r="C31" s="15">
-        <v>0.011930693069306941</v>
+        <v>0.0050000000000000044</v>
       </c>
       <c r="D31" s="15">
-        <v>0.07193069306930694</v>
+        <v>0.065</v>
       </c>
       <c r="E31" s="15">
         <v>0.03</v>
@@ -2885,16 +2888,16 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="12">
-        <v>44343</v>
+        <v>44315</v>
       </c>
       <c r="B32" s="15">
         <v>0</v>
       </c>
       <c r="C32" s="15">
-        <v>0.01726586102719034</v>
+        <v>0.011930693069306941</v>
       </c>
       <c r="D32" s="15">
-        <v>0.07726586102719034</v>
+        <v>0.07193069306930694</v>
       </c>
       <c r="E32" s="15">
         <v>0.03</v>
@@ -2905,36 +2908,36 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="12">
-        <v>44371</v>
+        <v>44343</v>
       </c>
       <c r="B33" s="15">
         <v>0</v>
       </c>
       <c r="C33" s="15">
-        <v>0.021768802228412265</v>
+        <v>0.01726586102719034</v>
       </c>
       <c r="D33" s="15">
-        <v>0.08176880222841226</v>
+        <v>0.07726586102719034</v>
       </c>
       <c r="E33" s="15">
         <v>0.03</v>
       </c>
       <c r="F33" s="15">
-        <v>0.0345</v>
+        <v>0.031</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="12">
-        <v>44406</v>
+        <v>44371</v>
       </c>
       <c r="B34" s="15">
         <v>0</v>
       </c>
       <c r="C34" s="15">
-        <v>0.026497461928934013</v>
+        <v>0.021768802228412265</v>
       </c>
       <c r="D34" s="15">
-        <v>0.08649746192893401</v>
+        <v>0.08176880222841226</v>
       </c>
       <c r="E34" s="15">
         <v>0.03</v>
@@ -2945,16 +2948,16 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="12">
-        <v>44434</v>
+        <v>44406</v>
       </c>
       <c r="B35" s="15">
         <v>0</v>
       </c>
       <c r="C35" s="15">
-        <v>0.029715639810426547</v>
+        <v>0.026497461928934013</v>
       </c>
       <c r="D35" s="15">
-        <v>0.08971563981042655</v>
+        <v>0.08649746192893401</v>
       </c>
       <c r="E35" s="15">
         <v>0.03</v>
@@ -2965,16 +2968,16 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="12">
-        <v>44469</v>
+        <v>44434</v>
       </c>
       <c r="B36" s="15">
         <v>0</v>
       </c>
       <c r="C36" s="15">
-        <v>0.033183807439824964</v>
+        <v>0.029715639810426547</v>
       </c>
       <c r="D36" s="15">
-        <v>0.09318380743982496</v>
+        <v>0.08971563981042655</v>
       </c>
       <c r="E36" s="15">
         <v>0.03</v>
@@ -2985,16 +2988,16 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="12">
-        <v>44497</v>
+        <v>44469</v>
       </c>
       <c r="B37" s="15">
         <v>0</v>
       </c>
       <c r="C37" s="15">
-        <v>0.035597938144329905</v>
+        <v>0.033183807439824964</v>
       </c>
       <c r="D37" s="15">
-        <v>0.0955979381443299</v>
+        <v>0.09318380743982496</v>
       </c>
       <c r="E37" s="15">
         <v>0.03</v>
@@ -3005,16 +3008,16 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="12">
-        <v>44525</v>
+        <v>44497</v>
       </c>
       <c r="B38" s="15">
         <v>0</v>
       </c>
       <c r="C38" s="15">
-        <v>0.037748538011695934</v>
+        <v>0.035597938144329905</v>
       </c>
       <c r="D38" s="15">
-        <v>0.09774853801169593</v>
+        <v>0.0955979381443299</v>
       </c>
       <c r="E38" s="15">
         <v>0.03</v>
@@ -3025,36 +3028,36 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="12">
-        <v>44560</v>
+        <v>44525</v>
       </c>
       <c r="B39" s="15">
         <v>0</v>
       </c>
       <c r="C39" s="15">
-        <v>0.04012773722627738</v>
+        <v>0.037748538011695934</v>
       </c>
       <c r="D39" s="15">
-        <v>0.10012773722627738</v>
+        <v>0.09774853801169593</v>
       </c>
       <c r="E39" s="15">
         <v>0.03</v>
       </c>
       <c r="F39" s="15">
-        <v>0.037000000000000005</v>
+        <v>0.0345</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="12">
-        <v>44588</v>
+        <v>44560</v>
       </c>
       <c r="B40" s="15">
         <v>0</v>
       </c>
       <c r="C40" s="15">
-        <v>0.04182291666666668</v>
+        <v>0.04012773722627738</v>
       </c>
       <c r="D40" s="15">
-        <v>0.10182291666666668</v>
+        <v>0.10012773722627738</v>
       </c>
       <c r="E40" s="15">
         <v>0.03</v>
@@ -3065,16 +3068,16 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="12">
-        <v>44616</v>
+        <v>44588</v>
       </c>
       <c r="B41" s="15">
         <v>0</v>
       </c>
       <c r="C41" s="15">
-        <v>0.04336092715231789</v>
+        <v>0.04182291666666668</v>
       </c>
       <c r="D41" s="15">
-        <v>0.10336092715231789</v>
+        <v>0.10182291666666668</v>
       </c>
       <c r="E41" s="15">
         <v>0.03</v>
@@ -3085,16 +3088,16 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="12">
-        <v>44651</v>
+        <v>44616</v>
       </c>
       <c r="B42" s="15">
         <v>0</v>
       </c>
       <c r="C42" s="15">
-        <v>0.04509389671361502</v>
+        <v>0.04336092715231789</v>
       </c>
       <c r="D42" s="15">
-        <v>0.10509389671361502</v>
+        <v>0.10336092715231789</v>
       </c>
       <c r="E42" s="15">
         <v>0.03</v>
@@ -3105,16 +3108,16 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="12">
-        <v>44679</v>
+        <v>44651</v>
       </c>
       <c r="B43" s="15">
         <v>0</v>
       </c>
       <c r="C43" s="15">
-        <v>0.04634932533733134</v>
+        <v>0.04509389671361502</v>
       </c>
       <c r="D43" s="15">
-        <v>0.10634932533733134</v>
+        <v>0.10509389671361502</v>
       </c>
       <c r="E43" s="15">
         <v>0.03</v>
@@ -3125,16 +3128,16 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="12">
-        <v>44707</v>
+        <v>44679</v>
       </c>
       <c r="B44" s="15">
         <v>0</v>
       </c>
       <c r="C44" s="15">
-        <v>0.04750359712230216</v>
+        <v>0.04634932533733134</v>
       </c>
       <c r="D44" s="15">
-        <v>0.10750359712230216</v>
+        <v>0.10634932533733134</v>
       </c>
       <c r="E44" s="15">
         <v>0.03</v>
@@ -3145,36 +3148,36 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="12">
-        <v>44742</v>
+        <v>44707</v>
       </c>
       <c r="B45" s="15">
         <v>0</v>
       </c>
       <c r="C45" s="15">
-        <v>0.04882191780821919</v>
+        <v>0.04750359712230216</v>
       </c>
       <c r="D45" s="15">
-        <v>0.10882191780821919</v>
+        <v>0.10750359712230216</v>
       </c>
       <c r="E45" s="15">
         <v>0.03</v>
       </c>
       <c r="F45" s="15">
-        <v>0.0385</v>
+        <v>0.037000000000000005</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="12">
-        <v>44770</v>
+        <v>44742</v>
       </c>
       <c r="B46" s="15">
         <v>0</v>
       </c>
       <c r="C46" s="15">
-        <v>0.049788918205804764</v>
+        <v>0.04882191780821919</v>
       </c>
       <c r="D46" s="15">
-        <v>0.10978891820580476</v>
+        <v>0.10882191780821919</v>
       </c>
       <c r="E46" s="15">
         <v>0.03</v>
@@ -3185,16 +3188,16 @@
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="12">
-        <v>44798</v>
+        <v>44770</v>
       </c>
       <c r="B47" s="15">
         <v>0</v>
       </c>
       <c r="C47" s="15">
-        <v>0.05068702290076338</v>
+        <v>0.049788918205804764</v>
       </c>
       <c r="D47" s="15">
-        <v>0.11068702290076338</v>
+        <v>0.10978891820580476</v>
       </c>
       <c r="E47" s="15">
         <v>0.03</v>
@@ -3205,16 +3208,16 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="12">
-        <v>44833</v>
+        <v>44798</v>
       </c>
       <c r="B48" s="15">
         <v>0</v>
       </c>
       <c r="C48" s="15">
-        <v>0.051723507917174186</v>
+        <v>0.05068702290076338</v>
       </c>
       <c r="D48" s="15">
-        <v>0.11172350791717418</v>
+        <v>0.11068702290076338</v>
       </c>
       <c r="E48" s="15">
         <v>0.03</v>
@@ -3225,16 +3228,16 @@
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="12">
-        <v>44861</v>
+        <v>44833</v>
       </c>
       <c r="B49" s="15">
         <v>0</v>
       </c>
       <c r="C49" s="15">
-        <v>0.05249116607773853</v>
+        <v>0.051723507917174186</v>
       </c>
       <c r="D49" s="15">
-        <v>0.11249116607773853</v>
+        <v>0.11172350791717418</v>
       </c>
       <c r="E49" s="15">
         <v>0.03</v>
@@ -3245,16 +3248,16 @@
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="12">
-        <v>44889</v>
+        <v>44861</v>
       </c>
       <c r="B50" s="15">
         <v>0</v>
       </c>
       <c r="C50" s="15">
-        <v>0.05320980615735463</v>
+        <v>0.05249116607773853</v>
       </c>
       <c r="D50" s="15">
-        <v>0.11320980615735463</v>
+        <v>0.11249116607773853</v>
       </c>
       <c r="E50" s="15">
         <v>0.03</v>
@@ -3265,36 +3268,36 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="12">
-        <v>44924</v>
+        <v>44889</v>
       </c>
       <c r="B51" s="15">
         <v>0</v>
       </c>
       <c r="C51" s="15">
-        <v>0.05404605263157895</v>
+        <v>0.05320980615735463</v>
       </c>
       <c r="D51" s="15">
-        <v>0.11404605263157895</v>
+        <v>0.11320980615735463</v>
       </c>
       <c r="E51" s="15">
         <v>0.03</v>
       </c>
       <c r="F51" s="15">
-        <v>0.0395</v>
+        <v>0.0385</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="12">
-        <v>44951</v>
+        <v>44924</v>
       </c>
       <c r="B52" s="15">
         <v>0</v>
       </c>
       <c r="C52" s="15">
-        <v>0.0546485623003195</v>
+        <v>0.05404605263157895</v>
       </c>
       <c r="D52" s="15">
-        <v>0.1146485623003195</v>
+        <v>0.11404605263157895</v>
       </c>
       <c r="E52" s="15">
         <v>0.03</v>
@@ -3305,16 +3308,16 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="12">
-        <v>44980</v>
+        <v>44951</v>
       </c>
       <c r="B53" s="15">
         <v>0</v>
       </c>
       <c r="C53" s="15">
-        <v>0.05525826446280993</v>
+        <v>0.0546485623003195</v>
       </c>
       <c r="D53" s="15">
-        <v>0.11525826446280993</v>
+        <v>0.1146485623003195</v>
       </c>
       <c r="E53" s="15">
         <v>0.03</v>
@@ -3325,16 +3328,16 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="12">
-        <v>45015</v>
+        <v>44980</v>
       </c>
       <c r="B54" s="15">
         <v>0</v>
       </c>
       <c r="C54" s="15">
-        <v>0.055947158524426735</v>
+        <v>0.05525826446280993</v>
       </c>
       <c r="D54" s="15">
-        <v>0.11594715852442673</v>
+        <v>0.11525826446280993</v>
       </c>
       <c r="E54" s="15">
         <v>0.03</v>
@@ -3345,16 +3348,16 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="12">
-        <v>45043</v>
+        <v>45015</v>
       </c>
       <c r="B55" s="15">
         <v>0</v>
       </c>
       <c r="C55" s="15">
-        <v>0.056464597478176545</v>
+        <v>0.055947158524426735</v>
       </c>
       <c r="D55" s="15">
-        <v>0.11646459747817654</v>
+        <v>0.11594715852442673</v>
       </c>
       <c r="E55" s="15">
         <v>0.03</v>
@@ -3365,16 +3368,16 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="12">
-        <v>45071</v>
+        <v>45043</v>
       </c>
       <c r="B56" s="15">
         <v>0</v>
       </c>
       <c r="C56" s="15">
-        <v>0.05695467422096319</v>
+        <v>0.056464597478176545</v>
       </c>
       <c r="D56" s="15">
-        <v>0.11695467422096319</v>
+        <v>0.11646459747817654</v>
       </c>
       <c r="E56" s="15">
         <v>0.03</v>
@@ -3385,36 +3388,36 @@
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="12">
-        <v>45106</v>
+        <v>45071</v>
       </c>
       <c r="B57" s="15">
         <v>0</v>
       </c>
       <c r="C57" s="15">
-        <v>0.05746788990825688</v>
+        <v>0.05695467422096319</v>
       </c>
       <c r="D57" s="15">
-        <v>0.11746788990825688</v>
+        <v>0.11695467422096319</v>
       </c>
       <c r="E57" s="15">
         <v>0.03</v>
       </c>
       <c r="F57" s="15">
-        <v>0.0445</v>
+        <v>0.0395</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="12">
-        <v>45134</v>
+        <v>45106</v>
       </c>
       <c r="B58" s="15">
         <v>0</v>
       </c>
       <c r="C58" s="15">
-        <v>0.05796791443850269</v>
+        <v>0.05746788990825688</v>
       </c>
       <c r="D58" s="15">
-        <v>0.11796791443850269</v>
+        <v>0.11746788990825688</v>
       </c>
       <c r="E58" s="15">
         <v>0.03</v>
@@ -3425,16 +3428,16 @@
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="12">
-        <v>45169</v>
+        <v>45134</v>
       </c>
       <c r="B59" s="15">
         <v>0</v>
       </c>
       <c r="C59" s="15">
-        <v>0.05848314606741574</v>
+        <v>0.05796791443850269</v>
       </c>
       <c r="D59" s="15">
-        <v>0.11848314606741574</v>
+        <v>0.11796791443850269</v>
       </c>
       <c r="E59" s="15">
         <v>0.03</v>
@@ -3445,16 +3448,16 @@
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="12">
-        <v>45197</v>
+        <v>45169</v>
       </c>
       <c r="B60" s="15">
         <v>0</v>
       </c>
       <c r="C60" s="15">
-        <v>0.058873417721518995</v>
+        <v>0.05848314606741574</v>
       </c>
       <c r="D60" s="15">
-        <v>0.11887341772151899</v>
+        <v>0.11848314606741574</v>
       </c>
       <c r="E60" s="15">
         <v>0.03</v>
@@ -3465,16 +3468,16 @@
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="12">
-        <v>45225</v>
+        <v>45197</v>
       </c>
       <c r="B61" s="15">
         <v>0</v>
       </c>
       <c r="C61" s="15">
-        <v>0.059245671887881296</v>
+        <v>0.058873417721518995</v>
       </c>
       <c r="D61" s="15">
-        <v>0.1192456718878813</v>
+        <v>0.11887341772151899</v>
       </c>
       <c r="E61" s="15">
         <v>0.03</v>
@@ -3485,16 +3488,16 @@
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="12">
-        <v>45260</v>
+        <v>45225</v>
       </c>
       <c r="B62" s="15">
         <v>0</v>
       </c>
       <c r="C62" s="15">
-        <v>0.059687500000000004</v>
+        <v>0.059245671887881296</v>
       </c>
       <c r="D62" s="15">
-        <v>0.1196875</v>
+        <v>0.1192456718878813</v>
       </c>
       <c r="E62" s="15">
         <v>0.03</v>
@@ -3505,16 +3508,16 @@
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="12">
-        <v>45288</v>
+        <v>45260</v>
       </c>
       <c r="B63" s="15">
         <v>0</v>
       </c>
       <c r="C63" s="15">
-        <v>0.060023510971786834</v>
+        <v>0.059687500000000004</v>
       </c>
       <c r="D63" s="15">
-        <v>0.12002351097178683</v>
+        <v>0.1196875</v>
       </c>
       <c r="E63" s="15">
         <v>0.03</v>
@@ -3525,7 +3528,7 @@
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="12">
-        <v>45316</v>
+        <v>45288</v>
       </c>
       <c r="B64" s="15">
         <v>0</v>
@@ -3545,7 +3548,7 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="12">
-        <v>45351</v>
+        <v>45316</v>
       </c>
       <c r="B65" s="15">
         <v>0</v>
@@ -3565,7 +3568,7 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="12">
-        <v>45687</v>
+        <v>45351</v>
       </c>
       <c r="B66" s="15">
         <v>0</v>
@@ -3585,16 +3588,16 @@
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="12">
-        <v>45715</v>
+        <v>45687</v>
       </c>
       <c r="B67" s="15">
         <v>0</v>
       </c>
       <c r="C67" s="15">
-        <v>0.060285605483625285</v>
+        <v>0.060023510971786834</v>
       </c>
       <c r="D67" s="15">
-        <v>0.12028560548362528</v>
+        <v>0.12002351097178683</v>
       </c>
       <c r="E67" s="15">
         <v>0.03</v>
@@ -3605,7 +3608,7 @@
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="12">
-        <v>45743</v>
+        <v>45715</v>
       </c>
       <c r="B68" s="15">
         <v>0</v>
@@ -3625,7 +3628,7 @@
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="12">
-        <v>45771</v>
+        <v>45743</v>
       </c>
       <c r="B69" s="15">
         <v>0</v>
@@ -3645,7 +3648,7 @@
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="12">
-        <v>45806</v>
+        <v>45771</v>
       </c>
       <c r="B70" s="15">
         <v>0</v>
@@ -3665,7 +3668,7 @@
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="12">
-        <v>45834</v>
+        <v>45806</v>
       </c>
       <c r="B71" s="15">
         <v>0</v>
@@ -3685,7 +3688,7 @@
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="12">
-        <v>45869</v>
+        <v>45834</v>
       </c>
       <c r="B72" s="15">
         <v>0</v>
@@ -3705,7 +3708,7 @@
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="12">
-        <v>45897</v>
+        <v>45869</v>
       </c>
       <c r="B73" s="15">
         <v>0</v>
@@ -3725,7 +3728,7 @@
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="12">
-        <v>45925</v>
+        <v>45897</v>
       </c>
       <c r="B74" s="15">
         <v>0</v>
@@ -3745,7 +3748,7 @@
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" s="12">
-        <v>45960</v>
+        <v>45925</v>
       </c>
       <c r="B75" s="15">
         <v>0</v>
@@ -3765,7 +3768,7 @@
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" s="12">
-        <v>45988</v>
+        <v>45960</v>
       </c>
       <c r="B76" s="15">
         <v>0</v>
@@ -3785,7 +3788,7 @@
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="12">
-        <v>46015</v>
+        <v>45988</v>
       </c>
       <c r="B77" s="15">
         <v>0</v>
@@ -3805,7 +3808,7 @@
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" s="12">
-        <v>46051</v>
+        <v>46015</v>
       </c>
       <c r="B78" s="15">
         <v>0</v>
@@ -3825,7 +3828,7 @@
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" s="12">
-        <v>46079</v>
+        <v>46051</v>
       </c>
       <c r="B79" s="15">
         <v>0</v>
@@ -3845,7 +3848,7 @@
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" s="12">
-        <v>46107</v>
+        <v>46079</v>
       </c>
       <c r="B80" s="15">
         <v>0</v>
@@ -3865,7 +3868,7 @@
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" s="12">
-        <v>46142</v>
+        <v>46107</v>
       </c>
       <c r="B81" s="15">
         <v>0</v>
@@ -3885,7 +3888,7 @@
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" s="12">
-        <v>46170</v>
+        <v>46142</v>
       </c>
       <c r="B82" s="15">
         <v>0</v>
@@ -3905,7 +3908,7 @@
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" s="12">
-        <v>46198</v>
+        <v>46170</v>
       </c>
       <c r="B83" s="15">
         <v>0</v>
@@ -3925,7 +3928,7 @@
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" s="12">
-        <v>46233</v>
+        <v>46198</v>
       </c>
       <c r="B84" s="15">
         <v>0</v>
@@ -3945,7 +3948,7 @@
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" s="12">
-        <v>46261</v>
+        <v>46233</v>
       </c>
       <c r="B85" s="15">
         <v>0</v>
@@ -3965,7 +3968,7 @@
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" s="12">
-        <v>46289</v>
+        <v>46261</v>
       </c>
       <c r="B86" s="15">
         <v>0</v>
@@ -3985,7 +3988,7 @@
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" s="12">
-        <v>46324</v>
+        <v>46289</v>
       </c>
       <c r="B87" s="15">
         <v>0</v>
@@ -4000,12 +4003,12 @@
         <v>0.03</v>
       </c>
       <c r="F87" s="15">
-        <v>0.055</v>
+        <v>0.0445</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" s="12">
-        <v>46352</v>
+        <v>46324</v>
       </c>
       <c r="B88" s="15">
         <v>0</v>
@@ -4025,7 +4028,7 @@
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" s="12">
-        <v>46387</v>
+        <v>46352</v>
       </c>
       <c r="B89" s="15">
         <v>0</v>
@@ -4045,7 +4048,7 @@
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" s="12">
-        <v>46415</v>
+        <v>46387</v>
       </c>
       <c r="B90" s="15">
         <v>0</v>
@@ -4065,7 +4068,7 @@
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" s="12">
-        <v>46443</v>
+        <v>46415</v>
       </c>
       <c r="B91" s="15">
         <v>0</v>
@@ -4085,7 +4088,7 @@
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" s="12">
-        <v>46471</v>
+        <v>46443</v>
       </c>
       <c r="B92" s="15">
         <v>0</v>
@@ -4125,7 +4128,7 @@
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" s="12">
-        <v>46506</v>
+        <v>46471</v>
       </c>
       <c r="B94" s="15">
         <v>0</v>
@@ -4145,7 +4148,7 @@
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" s="12">
-        <v>46534</v>
+        <v>46506</v>
       </c>
       <c r="B95" s="15">
         <v>0</v>
@@ -4165,7 +4168,7 @@
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" s="12">
-        <v>46562</v>
+        <v>46534</v>
       </c>
       <c r="B96" s="15">
         <v>0</v>
@@ -4185,7 +4188,7 @@
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" s="12">
-        <v>46597</v>
+        <v>46562</v>
       </c>
       <c r="B97" s="15">
         <v>0</v>
@@ -4205,7 +4208,7 @@
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" s="12">
-        <v>46625</v>
+        <v>46597</v>
       </c>
       <c r="B98" s="15">
         <v>0</v>
@@ -4225,7 +4228,7 @@
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" s="12">
-        <v>46660</v>
+        <v>46625</v>
       </c>
       <c r="B99" s="15">
         <v>0</v>
@@ -4245,7 +4248,7 @@
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" s="12">
-        <v>46688</v>
+        <v>46660</v>
       </c>
       <c r="B100" s="15">
         <v>0</v>
@@ -4265,7 +4268,7 @@
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="12">
-        <v>46716</v>
+        <v>46688</v>
       </c>
       <c r="B101" s="15">
         <v>0</v>
@@ -4285,7 +4288,7 @@
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102" s="12">
-        <v>46751</v>
+        <v>46716</v>
       </c>
       <c r="B102" s="15">
         <v>0</v>
@@ -4305,7 +4308,7 @@
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103" s="12">
-        <v>46779</v>
+        <v>46751</v>
       </c>
       <c r="B103" s="15">
         <v>0</v>
@@ -4325,7 +4328,7 @@
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104" s="12">
-        <v>46807</v>
+        <v>46779</v>
       </c>
       <c r="B104" s="15">
         <v>0</v>
@@ -4345,7 +4348,7 @@
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105" s="12">
-        <v>46842</v>
+        <v>46807</v>
       </c>
       <c r="B105" s="15">
         <v>0</v>
@@ -4365,7 +4368,7 @@
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106" s="12">
-        <v>46870</v>
+        <v>46842</v>
       </c>
       <c r="B106" s="15">
         <v>0</v>
@@ -4385,7 +4388,7 @@
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107" s="12">
-        <v>46898</v>
+        <v>46870</v>
       </c>
       <c r="B107" s="15">
         <v>0</v>
@@ -4405,7 +4408,7 @@
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108" s="12">
-        <v>46933</v>
+        <v>46898</v>
       </c>
       <c r="B108" s="15">
         <v>0</v>
@@ -4425,7 +4428,7 @@
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109" s="12">
-        <v>46959</v>
+        <v>46933</v>
       </c>
       <c r="B109" s="15">
         <v>0</v>
@@ -4445,7 +4448,7 @@
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110" s="12">
-        <v>46994</v>
+        <v>46959</v>
       </c>
       <c r="B110" s="15">
         <v>0</v>
@@ -4465,7 +4468,7 @@
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111" s="12">
-        <v>47022</v>
+        <v>46994</v>
       </c>
       <c r="B111" s="15">
         <v>0</v>
@@ -4485,7 +4488,7 @@
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112" s="12">
-        <v>47052</v>
+        <v>47022</v>
       </c>
       <c r="B112" s="15">
         <v>0</v>
@@ -4505,7 +4508,7 @@
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113" s="12">
-        <v>47087</v>
+        <v>47052</v>
       </c>
       <c r="B113" s="15">
         <v>0</v>
@@ -4525,7 +4528,7 @@
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A114" s="12">
-        <v>47115</v>
+        <v>47087</v>
       </c>
       <c r="B114" s="15">
         <v>0</v>
@@ -4545,7 +4548,7 @@
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115" s="12">
-        <v>47143</v>
+        <v>47115</v>
       </c>
       <c r="B115" s="15">
         <v>0</v>
@@ -4565,7 +4568,7 @@
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A116" s="12">
-        <v>47171</v>
+        <v>47143</v>
       </c>
       <c r="B116" s="15">
         <v>0</v>
@@ -4585,7 +4588,7 @@
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A117" s="12">
-        <v>47206</v>
+        <v>47171</v>
       </c>
       <c r="B117" s="15">
         <v>0</v>
@@ -4605,7 +4608,7 @@
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A118" s="12">
-        <v>47234</v>
+        <v>47206</v>
       </c>
       <c r="B118" s="15">
         <v>0</v>
@@ -4625,7 +4628,7 @@
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A119" s="12">
-        <v>47269</v>
+        <v>47234</v>
       </c>
       <c r="B119" s="15">
         <v>0</v>
@@ -4645,7 +4648,7 @@
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A120" s="12">
-        <v>47297</v>
+        <v>47269</v>
       </c>
       <c r="B120" s="15">
         <v>0</v>
@@ -4665,7 +4668,7 @@
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A121" s="12">
-        <v>47325</v>
+        <v>47297</v>
       </c>
       <c r="B121" s="15">
         <v>0</v>
@@ -4685,7 +4688,7 @@
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A122" s="12">
-        <v>47360</v>
+        <v>47325</v>
       </c>
       <c r="B122" s="15">
         <v>0</v>
@@ -4705,7 +4708,7 @@
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A123" s="12">
-        <v>47388</v>
+        <v>47360</v>
       </c>
       <c r="B123" s="15">
         <v>0</v>
@@ -4725,7 +4728,7 @@
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A124" s="12">
-        <v>47416</v>
+        <v>47388</v>
       </c>
       <c r="B124" s="15">
         <v>0</v>
@@ -4745,7 +4748,7 @@
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A125" s="12">
-        <v>47451</v>
+        <v>47416</v>
       </c>
       <c r="B125" s="15">
         <v>0</v>
@@ -4765,7 +4768,7 @@
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A126" s="12">
-        <v>47479</v>
+        <v>47451</v>
       </c>
       <c r="B126" s="15">
         <v>0</v>
@@ -4785,7 +4788,7 @@
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A127" s="12">
-        <v>47514</v>
+        <v>47479</v>
       </c>
       <c r="B127" s="15">
         <v>0</v>
@@ -4805,7 +4808,7 @@
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A128" s="12">
-        <v>47542</v>
+        <v>47514</v>
       </c>
       <c r="B128" s="15">
         <v>0</v>
@@ -4825,7 +4828,7 @@
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A129" s="12">
-        <v>47570</v>
+        <v>47542</v>
       </c>
       <c r="B129" s="15">
         <v>0</v>
@@ -4845,7 +4848,7 @@
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A130" s="12">
-        <v>47598</v>
+        <v>47570</v>
       </c>
       <c r="B130" s="15">
         <v>0</v>
@@ -4865,7 +4868,7 @@
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A131" s="12">
-        <v>47633</v>
+        <v>47598</v>
       </c>
       <c r="B131" s="15">
         <v>0</v>
@@ -4885,7 +4888,7 @@
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A132" s="12">
-        <v>47661</v>
+        <v>47633</v>
       </c>
       <c r="B132" s="15">
         <v>0</v>
@@ -4905,7 +4908,7 @@
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A133" s="12">
-        <v>47689</v>
+        <v>47661</v>
       </c>
       <c r="B133" s="15">
         <v>0</v>
@@ -4925,7 +4928,7 @@
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A134" s="12">
-        <v>47724</v>
+        <v>47689</v>
       </c>
       <c r="B134" s="15">
         <v>0</v>
@@ -4945,7 +4948,7 @@
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A135" s="12">
-        <v>47752</v>
+        <v>47724</v>
       </c>
       <c r="B135" s="15">
         <v>0</v>
@@ -4965,7 +4968,7 @@
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A136" s="12">
-        <v>47787</v>
+        <v>47752</v>
       </c>
       <c r="B136" s="15">
         <v>0</v>
@@ -4985,7 +4988,7 @@
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A137" s="12">
-        <v>47815</v>
+        <v>47787</v>
       </c>
       <c r="B137" s="15">
         <v>0</v>
@@ -5005,7 +5008,7 @@
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A138" s="12">
-        <v>47843</v>
+        <v>47815</v>
       </c>
       <c r="B138" s="15">
         <v>0</v>
@@ -5025,7 +5028,7 @@
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A139" s="12">
-        <v>47878</v>
+        <v>47843</v>
       </c>
       <c r="B139" s="15">
         <v>0</v>
@@ -5045,7 +5048,7 @@
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A140" s="12">
-        <v>47906</v>
+        <v>47878</v>
       </c>
       <c r="B140" s="15">
         <v>0</v>
@@ -5065,7 +5068,7 @@
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A141" s="12">
-        <v>47934</v>
+        <v>47906</v>
       </c>
       <c r="B141" s="15">
         <v>0</v>
@@ -5085,21 +5088,41 @@
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A142" s="12">
+        <v>47934</v>
+      </c>
+      <c r="B142" s="15">
+        <v>0</v>
+      </c>
+      <c r="C142" s="15">
+        <v>0.060285605483625285</v>
+      </c>
+      <c r="D142" s="15">
+        <v>0.12028560548362528</v>
+      </c>
+      <c r="E142" s="15">
+        <v>0.03</v>
+      </c>
+      <c r="F142" s="15">
+        <v>0.055</v>
+      </c>
+    </row>
+    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A143" s="12">
         <v>47962</v>
       </c>
-      <c r="B142" s="15">
-        <v>0</v>
-      </c>
-      <c r="C142" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D142" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E142" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F142" s="15">
+      <c r="B143" s="15">
+        <v>0</v>
+      </c>
+      <c r="C143" s="15">
+        <v>0.060285605483625285</v>
+      </c>
+      <c r="D143" s="15">
+        <v>0.12028560548362528</v>
+      </c>
+      <c r="E143" s="15">
+        <v>0.03</v>
+      </c>
+      <c r="F143" s="15">
         <v>0.055</v>
       </c>
     </row>
@@ -5118,11 +5141,12 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="30" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5167,7 +5191,7 @@
     </row>
     <row r="5" ht="36" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -5179,7 +5203,7 @@
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
@@ -5202,84 +5226,92 @@
       <c r="H7" s="5"/>
     </row>
     <row r="8" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="12">
-        <v>44196</v>
+        <v>31</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="13">
+        <v>0</v>
       </c>
       <c r="B10" s="13">
-        <v>4.198386446081097</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="12">
-        <v>44280</v>
+        <v>6.5</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="13">
+        <v>1</v>
       </c>
       <c r="B11" s="13">
-        <v>4.259978722050547</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="12">
-        <v>44371</v>
+        <v>6.5</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="13">
+        <v>2</v>
       </c>
       <c r="B12" s="13">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="12">
-        <v>44560</v>
+        <v>6.5</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="13">
+        <v>3</v>
       </c>
       <c r="B13" s="13">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="12">
-        <v>44742</v>
+        <v>6.5</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="13">
+        <v>5</v>
       </c>
       <c r="B14" s="13">
-        <v>4.579999999999999</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="12">
-        <v>44924</v>
+        <v>6.5</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="13">
+        <v>7</v>
       </c>
       <c r="B15" s="13">
-        <v>4.579999999999999</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="12">
-        <v>45105</v>
+        <v>6.5</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="13">
+        <v>10</v>
       </c>
       <c r="B16" s="13">
         <v>6.5</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="12">
-        <v>45288</v>
-      </c>
-      <c r="B17" s="13">
-        <v>6.5</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="12">
-        <v>46021</v>
-      </c>
-      <c r="B18" s="13">
-        <v>6.5</v>
+      <c r="C16" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -5346,7 +5378,7 @@
     </row>
     <row r="5" ht="36" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -5358,7 +5390,7 @@
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
@@ -5383,10 +5415,10 @@
     <row r="8" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Market data: forward grid, future dividends, per month surface parameters, surface toolbar
- Surface Parameters editor with Bid or Offer, Pricing Params scalars, both rate caps and the curve, saved per month with Reset
- Edit Surface, Upload Surface and Download Surface toolbar; cell validation; past expiry rows hidden
- Download Surface and the sample share one builder in the upload layout
- labels follow the underlying

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/samples/Hedging_Sheet_Vol_Surface_Sample.xlsx
+++ b/public/samples/Hedging_Sheet_Vol_Surface_Sample.xlsx
@@ -14,12 +14,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="36">
   <si>
-    <t>Volatility Surface Input · October 2026</t>
+    <t>October 2026 Volatility Surface</t>
   </si>
   <si>
-    <t>Implied volatility in percent points by strike and expiry. Strike rows are live formulas of the reference prices times the Strike Change.</t>
+    <t>Implied volatility in % points by strike and expiry. Strike rows are the reference prices times the Strike Change.</t>
   </si>
   <si>
     <t>Anand Rathi Wealth · Hedging Sheet</t>
@@ -43,7 +43,7 @@
     <t>Surface Parameters · October 2026</t>
   </si>
   <si>
-    <t>Reference prices are the 100 percent anchors of the Strike Change columns. The Pricing Params table is read by expiry date.</t>
+    <t>Reference prices are the 100% anchors of the Strike Change columns. The Pricing Params grid is read by expiry date.</t>
   </si>
   <si>
     <t>Parameter</t>
@@ -64,31 +64,31 @@
     <t>Reference Sensex Price</t>
   </si>
   <si>
+    <t>Bid or Offer</t>
+  </si>
+  <si>
+    <t>Bid</t>
+  </si>
+  <si>
     <t>Volatility Bump</t>
   </si>
   <si>
     <t>Forward Sell Rate</t>
   </si>
   <si>
+    <t>Dividend Bid or Offer Factor</t>
+  </si>
+  <si>
     <t>Rate Cap While Buying Forward</t>
   </si>
   <si>
-    <t>Dividend Bid Offer Multiplier</t>
-  </si>
-  <si>
-    <t>Bid or Offer</t>
-  </si>
-  <si>
-    <t>Bid</t>
+    <t>Rate Cap While Selling Forward</t>
   </si>
   <si>
     <t>Date</t>
   </si>
   <si>
-    <t>BID</t>
-  </si>
-  <si>
-    <t>Inc. Margin</t>
+    <t>Incremental Margin</t>
   </si>
   <si>
     <t>Full Margin</t>
@@ -97,19 +97,16 @@
     <t>Margin Cost</t>
   </si>
   <si>
-    <t>Fwd Sell rate</t>
-  </si>
-  <si>
     <t>Rate Curve</t>
   </si>
   <si>
-    <t>Tenors in years from the valuation date, with rates in percent per annum. Linked points follow the Premium Growth Rate.</t>
+    <t>Tenors in years from the valuation date, with rates in % per annum. Linked points follow the Premium Growth Rate.</t>
   </si>
   <si>
     <t>Tenor In Years</t>
   </si>
   <si>
-    <t>Rate In Percent</t>
+    <t>Rate %</t>
   </si>
   <si>
     <t>Linked To Premium Growth Rate</t>
@@ -121,10 +118,10 @@
     <t>Implied Dividends</t>
   </si>
   <si>
-    <t>Monthly implied dividends in Sensex index points.</t>
+    <t>Future implied dividends in Sensex index points. Nifty scales them by the ratio of the reference prices.</t>
   </si>
   <si>
-    <t>Implied Dividend</t>
+    <t>Implied Dividend In Index Points</t>
   </si>
 </sst>
 </file>
@@ -2489,12 +2486,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H143"/>
+  <dimension ref="A1:H77"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="6" width="14" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2610,29 +2609,29 @@
       <c r="A13" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="15">
-        <v>0</v>
+      <c r="B13" s="14" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B14" s="15">
-        <v>0.055</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B15" s="15">
-        <v>0.068</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B16" s="13">
         <v>1</v>
@@ -2640,975 +2639,963 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="B17" s="14" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="6" t="s">
+      <c r="B17" s="15">
+        <v>0.068</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B18" s="15">
+        <v>0.065</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="B21" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C21" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="D20" s="6" t="s">
+      <c r="D21" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="E20" s="6" t="s">
+      <c r="E21" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F20" s="6" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="12">
-        <v>43916</v>
-      </c>
-      <c r="B21" s="15">
-        <v>0</v>
-      </c>
-      <c r="C21" s="15">
-        <v>0.0050000000000000044</v>
-      </c>
-      <c r="D21" s="15">
-        <v>0.065</v>
-      </c>
-      <c r="E21" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F21" s="15">
-        <v>0</v>
+      <c r="F21" s="6" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="12">
-        <v>44007</v>
+        <v>46324</v>
       </c>
       <c r="B22" s="15">
         <v>0</v>
       </c>
       <c r="C22" s="15">
-        <v>0.0050000000000000044</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D22" s="15">
-        <v>0.065</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E22" s="15">
         <v>0.03</v>
       </c>
       <c r="F22" s="15">
-        <v>0</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="12">
-        <v>44042</v>
+        <v>46352</v>
       </c>
       <c r="B23" s="15">
         <v>0</v>
       </c>
       <c r="C23" s="15">
-        <v>0.0050000000000000044</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D23" s="15">
-        <v>0.065</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E23" s="15">
         <v>0.03</v>
       </c>
       <c r="F23" s="15">
-        <v>0</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="12">
-        <v>44070</v>
+        <v>46387</v>
       </c>
       <c r="B24" s="15">
         <v>0</v>
       </c>
       <c r="C24" s="15">
-        <v>0.0050000000000000044</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D24" s="15">
-        <v>0.065</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E24" s="15">
         <v>0.03</v>
       </c>
       <c r="F24" s="15">
-        <v>0.001</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="12">
-        <v>44098</v>
+        <v>46415</v>
       </c>
       <c r="B25" s="15">
         <v>0</v>
       </c>
       <c r="C25" s="15">
-        <v>0.0050000000000000044</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D25" s="15">
-        <v>0.065</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E25" s="15">
         <v>0.03</v>
       </c>
       <c r="F25" s="15">
-        <v>0.001</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="12">
-        <v>44133</v>
+        <v>46443</v>
       </c>
       <c r="B26" s="15">
         <v>0</v>
       </c>
       <c r="C26" s="15">
-        <v>0.0050000000000000044</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D26" s="15">
-        <v>0.065</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E26" s="15">
         <v>0.03</v>
       </c>
       <c r="F26" s="15">
-        <v>0.006</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="12">
-        <v>44160</v>
+        <v>46471</v>
       </c>
       <c r="B27" s="15">
         <v>0</v>
       </c>
       <c r="C27" s="15">
-        <v>0.0050000000000000044</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D27" s="15">
-        <v>0.065</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E27" s="15">
         <v>0.03</v>
       </c>
       <c r="F27" s="15">
-        <v>0.006</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="12">
-        <v>44196</v>
+        <v>46471</v>
       </c>
       <c r="B28" s="15">
         <v>0</v>
       </c>
       <c r="C28" s="15">
-        <v>0.0050000000000000044</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D28" s="15">
-        <v>0.065</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E28" s="15">
         <v>0.03</v>
       </c>
       <c r="F28" s="15">
-        <v>0.0085</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="12">
-        <v>44224</v>
+        <v>46506</v>
       </c>
       <c r="B29" s="15">
         <v>0</v>
       </c>
       <c r="C29" s="15">
-        <v>0.0050000000000000044</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D29" s="15">
-        <v>0.065</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E29" s="15">
         <v>0.03</v>
       </c>
       <c r="F29" s="15">
-        <v>0.0085</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="12">
-        <v>44252</v>
+        <v>46534</v>
       </c>
       <c r="B30" s="15">
         <v>0</v>
       </c>
       <c r="C30" s="15">
-        <v>0.0050000000000000044</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D30" s="15">
-        <v>0.065</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E30" s="15">
         <v>0.03</v>
       </c>
       <c r="F30" s="15">
-        <v>0.0085</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="12">
-        <v>44280</v>
+        <v>46562</v>
       </c>
       <c r="B31" s="15">
         <v>0</v>
       </c>
       <c r="C31" s="15">
-        <v>0.0050000000000000044</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D31" s="15">
-        <v>0.065</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E31" s="15">
         <v>0.03</v>
       </c>
       <c r="F31" s="15">
-        <v>0.031</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="12">
-        <v>44315</v>
+        <v>46597</v>
       </c>
       <c r="B32" s="15">
         <v>0</v>
       </c>
       <c r="C32" s="15">
-        <v>0.011930693069306941</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D32" s="15">
-        <v>0.07193069306930694</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E32" s="15">
         <v>0.03</v>
       </c>
       <c r="F32" s="15">
-        <v>0.031</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="12">
-        <v>44343</v>
+        <v>46625</v>
       </c>
       <c r="B33" s="15">
         <v>0</v>
       </c>
       <c r="C33" s="15">
-        <v>0.01726586102719034</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D33" s="15">
-        <v>0.07726586102719034</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E33" s="15">
         <v>0.03</v>
       </c>
       <c r="F33" s="15">
-        <v>0.031</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="12">
-        <v>44371</v>
+        <v>46660</v>
       </c>
       <c r="B34" s="15">
         <v>0</v>
       </c>
       <c r="C34" s="15">
-        <v>0.021768802228412265</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D34" s="15">
-        <v>0.08176880222841226</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E34" s="15">
         <v>0.03</v>
       </c>
       <c r="F34" s="15">
-        <v>0.0345</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="12">
-        <v>44406</v>
+        <v>46688</v>
       </c>
       <c r="B35" s="15">
         <v>0</v>
       </c>
       <c r="C35" s="15">
-        <v>0.026497461928934013</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D35" s="15">
-        <v>0.08649746192893401</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E35" s="15">
         <v>0.03</v>
       </c>
       <c r="F35" s="15">
-        <v>0.0345</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="12">
-        <v>44434</v>
+        <v>46716</v>
       </c>
       <c r="B36" s="15">
         <v>0</v>
       </c>
       <c r="C36" s="15">
-        <v>0.029715639810426547</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D36" s="15">
-        <v>0.08971563981042655</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E36" s="15">
         <v>0.03</v>
       </c>
       <c r="F36" s="15">
-        <v>0.0345</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="12">
-        <v>44469</v>
+        <v>46751</v>
       </c>
       <c r="B37" s="15">
         <v>0</v>
       </c>
       <c r="C37" s="15">
-        <v>0.033183807439824964</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D37" s="15">
-        <v>0.09318380743982496</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E37" s="15">
         <v>0.03</v>
       </c>
       <c r="F37" s="15">
-        <v>0.0345</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="12">
-        <v>44497</v>
+        <v>46779</v>
       </c>
       <c r="B38" s="15">
         <v>0</v>
       </c>
       <c r="C38" s="15">
-        <v>0.035597938144329905</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D38" s="15">
-        <v>0.0955979381443299</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E38" s="15">
         <v>0.03</v>
       </c>
       <c r="F38" s="15">
-        <v>0.0345</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="12">
-        <v>44525</v>
+        <v>46807</v>
       </c>
       <c r="B39" s="15">
         <v>0</v>
       </c>
       <c r="C39" s="15">
-        <v>0.037748538011695934</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D39" s="15">
-        <v>0.09774853801169593</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E39" s="15">
         <v>0.03</v>
       </c>
       <c r="F39" s="15">
-        <v>0.0345</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="12">
-        <v>44560</v>
+        <v>46842</v>
       </c>
       <c r="B40" s="15">
         <v>0</v>
       </c>
       <c r="C40" s="15">
-        <v>0.04012773722627738</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D40" s="15">
-        <v>0.10012773722627738</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E40" s="15">
         <v>0.03</v>
       </c>
       <c r="F40" s="15">
-        <v>0.037000000000000005</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="12">
-        <v>44588</v>
+        <v>46870</v>
       </c>
       <c r="B41" s="15">
         <v>0</v>
       </c>
       <c r="C41" s="15">
-        <v>0.04182291666666668</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D41" s="15">
-        <v>0.10182291666666668</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E41" s="15">
         <v>0.03</v>
       </c>
       <c r="F41" s="15">
-        <v>0.037000000000000005</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="12">
-        <v>44616</v>
+        <v>46898</v>
       </c>
       <c r="B42" s="15">
         <v>0</v>
       </c>
       <c r="C42" s="15">
-        <v>0.04336092715231789</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D42" s="15">
-        <v>0.10336092715231789</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E42" s="15">
         <v>0.03</v>
       </c>
       <c r="F42" s="15">
-        <v>0.037000000000000005</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="12">
-        <v>44651</v>
+        <v>46933</v>
       </c>
       <c r="B43" s="15">
         <v>0</v>
       </c>
       <c r="C43" s="15">
-        <v>0.04509389671361502</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D43" s="15">
-        <v>0.10509389671361502</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E43" s="15">
         <v>0.03</v>
       </c>
       <c r="F43" s="15">
-        <v>0.037000000000000005</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="12">
-        <v>44679</v>
+        <v>46959</v>
       </c>
       <c r="B44" s="15">
         <v>0</v>
       </c>
       <c r="C44" s="15">
-        <v>0.04634932533733134</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D44" s="15">
-        <v>0.10634932533733134</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E44" s="15">
         <v>0.03</v>
       </c>
       <c r="F44" s="15">
-        <v>0.037000000000000005</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="12">
-        <v>44707</v>
+        <v>46994</v>
       </c>
       <c r="B45" s="15">
         <v>0</v>
       </c>
       <c r="C45" s="15">
-        <v>0.04750359712230216</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D45" s="15">
-        <v>0.10750359712230216</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E45" s="15">
         <v>0.03</v>
       </c>
       <c r="F45" s="15">
-        <v>0.037000000000000005</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="12">
-        <v>44742</v>
+        <v>47022</v>
       </c>
       <c r="B46" s="15">
         <v>0</v>
       </c>
       <c r="C46" s="15">
-        <v>0.04882191780821919</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D46" s="15">
-        <v>0.10882191780821919</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E46" s="15">
         <v>0.03</v>
       </c>
       <c r="F46" s="15">
-        <v>0.0385</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="12">
-        <v>44770</v>
+        <v>47052</v>
       </c>
       <c r="B47" s="15">
         <v>0</v>
       </c>
       <c r="C47" s="15">
-        <v>0.049788918205804764</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D47" s="15">
-        <v>0.10978891820580476</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E47" s="15">
         <v>0.03</v>
       </c>
       <c r="F47" s="15">
-        <v>0.0385</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="12">
-        <v>44798</v>
+        <v>47087</v>
       </c>
       <c r="B48" s="15">
         <v>0</v>
       </c>
       <c r="C48" s="15">
-        <v>0.05068702290076338</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D48" s="15">
-        <v>0.11068702290076338</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E48" s="15">
         <v>0.03</v>
       </c>
       <c r="F48" s="15">
-        <v>0.0385</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="12">
-        <v>44833</v>
+        <v>47115</v>
       </c>
       <c r="B49" s="15">
         <v>0</v>
       </c>
       <c r="C49" s="15">
-        <v>0.051723507917174186</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D49" s="15">
-        <v>0.11172350791717418</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E49" s="15">
         <v>0.03</v>
       </c>
       <c r="F49" s="15">
-        <v>0.0385</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="12">
-        <v>44861</v>
+        <v>47143</v>
       </c>
       <c r="B50" s="15">
         <v>0</v>
       </c>
       <c r="C50" s="15">
-        <v>0.05249116607773853</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D50" s="15">
-        <v>0.11249116607773853</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E50" s="15">
         <v>0.03</v>
       </c>
       <c r="F50" s="15">
-        <v>0.0385</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="12">
-        <v>44889</v>
+        <v>47171</v>
       </c>
       <c r="B51" s="15">
         <v>0</v>
       </c>
       <c r="C51" s="15">
-        <v>0.05320980615735463</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D51" s="15">
-        <v>0.11320980615735463</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E51" s="15">
         <v>0.03</v>
       </c>
       <c r="F51" s="15">
-        <v>0.0385</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="12">
-        <v>44924</v>
+        <v>47206</v>
       </c>
       <c r="B52" s="15">
         <v>0</v>
       </c>
       <c r="C52" s="15">
-        <v>0.05404605263157895</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D52" s="15">
-        <v>0.11404605263157895</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E52" s="15">
         <v>0.03</v>
       </c>
       <c r="F52" s="15">
-        <v>0.0395</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="12">
-        <v>44951</v>
+        <v>47234</v>
       </c>
       <c r="B53" s="15">
         <v>0</v>
       </c>
       <c r="C53" s="15">
-        <v>0.0546485623003195</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D53" s="15">
-        <v>0.1146485623003195</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E53" s="15">
         <v>0.03</v>
       </c>
       <c r="F53" s="15">
-        <v>0.0395</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="12">
-        <v>44980</v>
+        <v>47269</v>
       </c>
       <c r="B54" s="15">
         <v>0</v>
       </c>
       <c r="C54" s="15">
-        <v>0.05525826446280993</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D54" s="15">
-        <v>0.11525826446280993</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E54" s="15">
         <v>0.03</v>
       </c>
       <c r="F54" s="15">
-        <v>0.0395</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="12">
-        <v>45015</v>
+        <v>47297</v>
       </c>
       <c r="B55" s="15">
         <v>0</v>
       </c>
       <c r="C55" s="15">
-        <v>0.055947158524426735</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D55" s="15">
-        <v>0.11594715852442673</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E55" s="15">
         <v>0.03</v>
       </c>
       <c r="F55" s="15">
-        <v>0.0395</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="12">
-        <v>45043</v>
+        <v>47325</v>
       </c>
       <c r="B56" s="15">
         <v>0</v>
       </c>
       <c r="C56" s="15">
-        <v>0.056464597478176545</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D56" s="15">
-        <v>0.11646459747817654</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E56" s="15">
         <v>0.03</v>
       </c>
       <c r="F56" s="15">
-        <v>0.0395</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="12">
-        <v>45071</v>
+        <v>47360</v>
       </c>
       <c r="B57" s="15">
         <v>0</v>
       </c>
       <c r="C57" s="15">
-        <v>0.05695467422096319</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D57" s="15">
-        <v>0.11695467422096319</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E57" s="15">
         <v>0.03</v>
       </c>
       <c r="F57" s="15">
-        <v>0.0395</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="12">
-        <v>45106</v>
+        <v>47388</v>
       </c>
       <c r="B58" s="15">
         <v>0</v>
       </c>
       <c r="C58" s="15">
-        <v>0.05746788990825688</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D58" s="15">
-        <v>0.11746788990825688</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E58" s="15">
         <v>0.03</v>
       </c>
       <c r="F58" s="15">
-        <v>0.0445</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="12">
-        <v>45134</v>
+        <v>47416</v>
       </c>
       <c r="B59" s="15">
         <v>0</v>
       </c>
       <c r="C59" s="15">
-        <v>0.05796791443850269</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D59" s="15">
-        <v>0.11796791443850269</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E59" s="15">
         <v>0.03</v>
       </c>
       <c r="F59" s="15">
-        <v>0.0445</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="12">
-        <v>45169</v>
+        <v>47451</v>
       </c>
       <c r="B60" s="15">
         <v>0</v>
       </c>
       <c r="C60" s="15">
-        <v>0.05848314606741574</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D60" s="15">
-        <v>0.11848314606741574</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E60" s="15">
         <v>0.03</v>
       </c>
       <c r="F60" s="15">
-        <v>0.0445</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="12">
-        <v>45197</v>
+        <v>47479</v>
       </c>
       <c r="B61" s="15">
         <v>0</v>
       </c>
       <c r="C61" s="15">
-        <v>0.058873417721518995</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D61" s="15">
-        <v>0.11887341772151899</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E61" s="15">
         <v>0.03</v>
       </c>
       <c r="F61" s="15">
-        <v>0.0445</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="12">
-        <v>45225</v>
+        <v>47514</v>
       </c>
       <c r="B62" s="15">
         <v>0</v>
       </c>
       <c r="C62" s="15">
-        <v>0.059245671887881296</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D62" s="15">
-        <v>0.1192456718878813</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E62" s="15">
         <v>0.03</v>
       </c>
       <c r="F62" s="15">
-        <v>0.0445</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="12">
-        <v>45260</v>
+        <v>47542</v>
       </c>
       <c r="B63" s="15">
         <v>0</v>
       </c>
       <c r="C63" s="15">
-        <v>0.059687500000000004</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D63" s="15">
-        <v>0.1196875</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E63" s="15">
         <v>0.03</v>
       </c>
       <c r="F63" s="15">
-        <v>0.0445</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="12">
-        <v>45288</v>
+        <v>47570</v>
       </c>
       <c r="B64" s="15">
         <v>0</v>
       </c>
       <c r="C64" s="15">
-        <v>0.060023510971786834</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D64" s="15">
-        <v>0.12002351097178683</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E64" s="15">
         <v>0.03</v>
       </c>
       <c r="F64" s="15">
-        <v>0.0445</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="12">
-        <v>45316</v>
+        <v>47598</v>
       </c>
       <c r="B65" s="15">
         <v>0</v>
       </c>
       <c r="C65" s="15">
-        <v>0.060023510971786834</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D65" s="15">
-        <v>0.12002351097178683</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E65" s="15">
         <v>0.03</v>
       </c>
       <c r="F65" s="15">
-        <v>0.0445</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="12">
-        <v>45351</v>
+        <v>47633</v>
       </c>
       <c r="B66" s="15">
         <v>0</v>
       </c>
       <c r="C66" s="15">
-        <v>0.060023510971786834</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D66" s="15">
-        <v>0.12002351097178683</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E66" s="15">
         <v>0.03</v>
       </c>
       <c r="F66" s="15">
-        <v>0.0445</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="12">
-        <v>45687</v>
+        <v>47661</v>
       </c>
       <c r="B67" s="15">
         <v>0</v>
       </c>
       <c r="C67" s="15">
-        <v>0.060023510971786834</v>
+        <v>0.060285605483625285</v>
       </c>
       <c r="D67" s="15">
-        <v>0.12002351097178683</v>
+        <v>0.12028560548362528</v>
       </c>
       <c r="E67" s="15">
         <v>0.03</v>
       </c>
       <c r="F67" s="15">
-        <v>0.0445</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="12">
-        <v>45715</v>
+        <v>47689</v>
       </c>
       <c r="B68" s="15">
         <v>0</v>
@@ -3623,12 +3610,12 @@
         <v>0.03</v>
       </c>
       <c r="F68" s="15">
-        <v>0.0445</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="12">
-        <v>45743</v>
+        <v>47724</v>
       </c>
       <c r="B69" s="15">
         <v>0</v>
@@ -3643,12 +3630,12 @@
         <v>0.03</v>
       </c>
       <c r="F69" s="15">
-        <v>0.0445</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="12">
-        <v>45771</v>
+        <v>47752</v>
       </c>
       <c r="B70" s="15">
         <v>0</v>
@@ -3663,12 +3650,12 @@
         <v>0.03</v>
       </c>
       <c r="F70" s="15">
-        <v>0.0445</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="12">
-        <v>45806</v>
+        <v>47787</v>
       </c>
       <c r="B71" s="15">
         <v>0</v>
@@ -3683,12 +3670,12 @@
         <v>0.03</v>
       </c>
       <c r="F71" s="15">
-        <v>0.0445</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="12">
-        <v>45834</v>
+        <v>47815</v>
       </c>
       <c r="B72" s="15">
         <v>0</v>
@@ -3703,12 +3690,12 @@
         <v>0.03</v>
       </c>
       <c r="F72" s="15">
-        <v>0.0445</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="12">
-        <v>45869</v>
+        <v>47843</v>
       </c>
       <c r="B73" s="15">
         <v>0</v>
@@ -3723,12 +3710,12 @@
         <v>0.03</v>
       </c>
       <c r="F73" s="15">
-        <v>0.0445</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="12">
-        <v>45897</v>
+        <v>47878</v>
       </c>
       <c r="B74" s="15">
         <v>0</v>
@@ -3743,12 +3730,12 @@
         <v>0.03</v>
       </c>
       <c r="F74" s="15">
-        <v>0.0445</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" s="12">
-        <v>45925</v>
+        <v>47906</v>
       </c>
       <c r="B75" s="15">
         <v>0</v>
@@ -3763,12 +3750,12 @@
         <v>0.03</v>
       </c>
       <c r="F75" s="15">
-        <v>0.0445</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" s="12">
-        <v>45960</v>
+        <v>47934</v>
       </c>
       <c r="B76" s="15">
         <v>0</v>
@@ -3783,12 +3770,12 @@
         <v>0.03</v>
       </c>
       <c r="F76" s="15">
-        <v>0.0445</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="12">
-        <v>45988</v>
+        <v>47962</v>
       </c>
       <c r="B77" s="15">
         <v>0</v>
@@ -3803,1326 +3790,6 @@
         <v>0.03</v>
       </c>
       <c r="F77" s="15">
-        <v>0.0445</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A78" s="12">
-        <v>46015</v>
-      </c>
-      <c r="B78" s="15">
-        <v>0</v>
-      </c>
-      <c r="C78" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D78" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E78" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F78" s="15">
-        <v>0.0445</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A79" s="12">
-        <v>46051</v>
-      </c>
-      <c r="B79" s="15">
-        <v>0</v>
-      </c>
-      <c r="C79" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D79" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E79" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F79" s="15">
-        <v>0.0445</v>
-      </c>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A80" s="12">
-        <v>46079</v>
-      </c>
-      <c r="B80" s="15">
-        <v>0</v>
-      </c>
-      <c r="C80" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D80" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E80" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F80" s="15">
-        <v>0.0445</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A81" s="12">
-        <v>46107</v>
-      </c>
-      <c r="B81" s="15">
-        <v>0</v>
-      </c>
-      <c r="C81" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D81" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E81" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F81" s="15">
-        <v>0.0445</v>
-      </c>
-    </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A82" s="12">
-        <v>46142</v>
-      </c>
-      <c r="B82" s="15">
-        <v>0</v>
-      </c>
-      <c r="C82" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D82" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E82" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F82" s="15">
-        <v>0.0445</v>
-      </c>
-    </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A83" s="12">
-        <v>46170</v>
-      </c>
-      <c r="B83" s="15">
-        <v>0</v>
-      </c>
-      <c r="C83" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D83" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E83" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F83" s="15">
-        <v>0.0445</v>
-      </c>
-    </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A84" s="12">
-        <v>46198</v>
-      </c>
-      <c r="B84" s="15">
-        <v>0</v>
-      </c>
-      <c r="C84" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D84" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E84" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F84" s="15">
-        <v>0.0445</v>
-      </c>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A85" s="12">
-        <v>46233</v>
-      </c>
-      <c r="B85" s="15">
-        <v>0</v>
-      </c>
-      <c r="C85" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D85" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E85" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F85" s="15">
-        <v>0.0445</v>
-      </c>
-    </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A86" s="12">
-        <v>46261</v>
-      </c>
-      <c r="B86" s="15">
-        <v>0</v>
-      </c>
-      <c r="C86" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D86" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E86" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F86" s="15">
-        <v>0.0445</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A87" s="12">
-        <v>46289</v>
-      </c>
-      <c r="B87" s="15">
-        <v>0</v>
-      </c>
-      <c r="C87" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D87" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E87" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F87" s="15">
-        <v>0.0445</v>
-      </c>
-    </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A88" s="12">
-        <v>46324</v>
-      </c>
-      <c r="B88" s="15">
-        <v>0</v>
-      </c>
-      <c r="C88" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D88" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E88" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F88" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A89" s="12">
-        <v>46352</v>
-      </c>
-      <c r="B89" s="15">
-        <v>0</v>
-      </c>
-      <c r="C89" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D89" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E89" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F89" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A90" s="12">
-        <v>46387</v>
-      </c>
-      <c r="B90" s="15">
-        <v>0</v>
-      </c>
-      <c r="C90" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D90" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E90" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F90" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A91" s="12">
-        <v>46415</v>
-      </c>
-      <c r="B91" s="15">
-        <v>0</v>
-      </c>
-      <c r="C91" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D91" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E91" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F91" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A92" s="12">
-        <v>46443</v>
-      </c>
-      <c r="B92" s="15">
-        <v>0</v>
-      </c>
-      <c r="C92" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D92" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E92" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F92" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A93" s="12">
-        <v>46471</v>
-      </c>
-      <c r="B93" s="15">
-        <v>0</v>
-      </c>
-      <c r="C93" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D93" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E93" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F93" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A94" s="12">
-        <v>46471</v>
-      </c>
-      <c r="B94" s="15">
-        <v>0</v>
-      </c>
-      <c r="C94" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D94" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E94" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F94" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A95" s="12">
-        <v>46506</v>
-      </c>
-      <c r="B95" s="15">
-        <v>0</v>
-      </c>
-      <c r="C95" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D95" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E95" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F95" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A96" s="12">
-        <v>46534</v>
-      </c>
-      <c r="B96" s="15">
-        <v>0</v>
-      </c>
-      <c r="C96" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D96" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E96" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F96" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A97" s="12">
-        <v>46562</v>
-      </c>
-      <c r="B97" s="15">
-        <v>0</v>
-      </c>
-      <c r="C97" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D97" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E97" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F97" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A98" s="12">
-        <v>46597</v>
-      </c>
-      <c r="B98" s="15">
-        <v>0</v>
-      </c>
-      <c r="C98" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D98" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E98" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F98" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A99" s="12">
-        <v>46625</v>
-      </c>
-      <c r="B99" s="15">
-        <v>0</v>
-      </c>
-      <c r="C99" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D99" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E99" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F99" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A100" s="12">
-        <v>46660</v>
-      </c>
-      <c r="B100" s="15">
-        <v>0</v>
-      </c>
-      <c r="C100" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D100" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E100" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F100" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A101" s="12">
-        <v>46688</v>
-      </c>
-      <c r="B101" s="15">
-        <v>0</v>
-      </c>
-      <c r="C101" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D101" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E101" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F101" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A102" s="12">
-        <v>46716</v>
-      </c>
-      <c r="B102" s="15">
-        <v>0</v>
-      </c>
-      <c r="C102" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D102" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E102" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F102" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A103" s="12">
-        <v>46751</v>
-      </c>
-      <c r="B103" s="15">
-        <v>0</v>
-      </c>
-      <c r="C103" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D103" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E103" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F103" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A104" s="12">
-        <v>46779</v>
-      </c>
-      <c r="B104" s="15">
-        <v>0</v>
-      </c>
-      <c r="C104" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D104" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E104" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F104" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A105" s="12">
-        <v>46807</v>
-      </c>
-      <c r="B105" s="15">
-        <v>0</v>
-      </c>
-      <c r="C105" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D105" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E105" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F105" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A106" s="12">
-        <v>46842</v>
-      </c>
-      <c r="B106" s="15">
-        <v>0</v>
-      </c>
-      <c r="C106" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D106" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E106" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F106" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A107" s="12">
-        <v>46870</v>
-      </c>
-      <c r="B107" s="15">
-        <v>0</v>
-      </c>
-      <c r="C107" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D107" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E107" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F107" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A108" s="12">
-        <v>46898</v>
-      </c>
-      <c r="B108" s="15">
-        <v>0</v>
-      </c>
-      <c r="C108" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D108" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E108" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F108" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A109" s="12">
-        <v>46933</v>
-      </c>
-      <c r="B109" s="15">
-        <v>0</v>
-      </c>
-      <c r="C109" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D109" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E109" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F109" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A110" s="12">
-        <v>46959</v>
-      </c>
-      <c r="B110" s="15">
-        <v>0</v>
-      </c>
-      <c r="C110" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D110" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E110" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F110" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A111" s="12">
-        <v>46994</v>
-      </c>
-      <c r="B111" s="15">
-        <v>0</v>
-      </c>
-      <c r="C111" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D111" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E111" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F111" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A112" s="12">
-        <v>47022</v>
-      </c>
-      <c r="B112" s="15">
-        <v>0</v>
-      </c>
-      <c r="C112" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D112" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E112" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F112" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A113" s="12">
-        <v>47052</v>
-      </c>
-      <c r="B113" s="15">
-        <v>0</v>
-      </c>
-      <c r="C113" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D113" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E113" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F113" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A114" s="12">
-        <v>47087</v>
-      </c>
-      <c r="B114" s="15">
-        <v>0</v>
-      </c>
-      <c r="C114" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D114" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E114" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F114" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A115" s="12">
-        <v>47115</v>
-      </c>
-      <c r="B115" s="15">
-        <v>0</v>
-      </c>
-      <c r="C115" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D115" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E115" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F115" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A116" s="12">
-        <v>47143</v>
-      </c>
-      <c r="B116" s="15">
-        <v>0</v>
-      </c>
-      <c r="C116" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D116" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E116" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F116" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A117" s="12">
-        <v>47171</v>
-      </c>
-      <c r="B117" s="15">
-        <v>0</v>
-      </c>
-      <c r="C117" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D117" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E117" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F117" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A118" s="12">
-        <v>47206</v>
-      </c>
-      <c r="B118" s="15">
-        <v>0</v>
-      </c>
-      <c r="C118" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D118" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E118" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F118" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A119" s="12">
-        <v>47234</v>
-      </c>
-      <c r="B119" s="15">
-        <v>0</v>
-      </c>
-      <c r="C119" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D119" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E119" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F119" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A120" s="12">
-        <v>47269</v>
-      </c>
-      <c r="B120" s="15">
-        <v>0</v>
-      </c>
-      <c r="C120" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D120" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E120" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F120" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A121" s="12">
-        <v>47297</v>
-      </c>
-      <c r="B121" s="15">
-        <v>0</v>
-      </c>
-      <c r="C121" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D121" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E121" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F121" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A122" s="12">
-        <v>47325</v>
-      </c>
-      <c r="B122" s="15">
-        <v>0</v>
-      </c>
-      <c r="C122" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D122" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E122" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F122" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A123" s="12">
-        <v>47360</v>
-      </c>
-      <c r="B123" s="15">
-        <v>0</v>
-      </c>
-      <c r="C123" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D123" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E123" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F123" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A124" s="12">
-        <v>47388</v>
-      </c>
-      <c r="B124" s="15">
-        <v>0</v>
-      </c>
-      <c r="C124" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D124" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E124" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F124" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A125" s="12">
-        <v>47416</v>
-      </c>
-      <c r="B125" s="15">
-        <v>0</v>
-      </c>
-      <c r="C125" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D125" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E125" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F125" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A126" s="12">
-        <v>47451</v>
-      </c>
-      <c r="B126" s="15">
-        <v>0</v>
-      </c>
-      <c r="C126" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D126" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E126" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F126" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A127" s="12">
-        <v>47479</v>
-      </c>
-      <c r="B127" s="15">
-        <v>0</v>
-      </c>
-      <c r="C127" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D127" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E127" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F127" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A128" s="12">
-        <v>47514</v>
-      </c>
-      <c r="B128" s="15">
-        <v>0</v>
-      </c>
-      <c r="C128" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D128" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E128" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F128" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A129" s="12">
-        <v>47542</v>
-      </c>
-      <c r="B129" s="15">
-        <v>0</v>
-      </c>
-      <c r="C129" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D129" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E129" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F129" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A130" s="12">
-        <v>47570</v>
-      </c>
-      <c r="B130" s="15">
-        <v>0</v>
-      </c>
-      <c r="C130" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D130" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E130" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F130" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A131" s="12">
-        <v>47598</v>
-      </c>
-      <c r="B131" s="15">
-        <v>0</v>
-      </c>
-      <c r="C131" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D131" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E131" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F131" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A132" s="12">
-        <v>47633</v>
-      </c>
-      <c r="B132" s="15">
-        <v>0</v>
-      </c>
-      <c r="C132" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D132" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E132" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F132" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A133" s="12">
-        <v>47661</v>
-      </c>
-      <c r="B133" s="15">
-        <v>0</v>
-      </c>
-      <c r="C133" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D133" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E133" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F133" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A134" s="12">
-        <v>47689</v>
-      </c>
-      <c r="B134" s="15">
-        <v>0</v>
-      </c>
-      <c r="C134" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D134" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E134" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F134" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A135" s="12">
-        <v>47724</v>
-      </c>
-      <c r="B135" s="15">
-        <v>0</v>
-      </c>
-      <c r="C135" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D135" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E135" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F135" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A136" s="12">
-        <v>47752</v>
-      </c>
-      <c r="B136" s="15">
-        <v>0</v>
-      </c>
-      <c r="C136" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D136" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E136" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F136" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A137" s="12">
-        <v>47787</v>
-      </c>
-      <c r="B137" s="15">
-        <v>0</v>
-      </c>
-      <c r="C137" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D137" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E137" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F137" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A138" s="12">
-        <v>47815</v>
-      </c>
-      <c r="B138" s="15">
-        <v>0</v>
-      </c>
-      <c r="C138" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D138" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E138" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F138" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A139" s="12">
-        <v>47843</v>
-      </c>
-      <c r="B139" s="15">
-        <v>0</v>
-      </c>
-      <c r="C139" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D139" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E139" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F139" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A140" s="12">
-        <v>47878</v>
-      </c>
-      <c r="B140" s="15">
-        <v>0</v>
-      </c>
-      <c r="C140" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D140" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E140" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F140" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A141" s="12">
-        <v>47906</v>
-      </c>
-      <c r="B141" s="15">
-        <v>0</v>
-      </c>
-      <c r="C141" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D141" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E141" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F141" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A142" s="12">
-        <v>47934</v>
-      </c>
-      <c r="B142" s="15">
-        <v>0</v>
-      </c>
-      <c r="C142" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D142" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E142" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F142" s="15">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A143" s="12">
-        <v>47962</v>
-      </c>
-      <c r="B143" s="15">
-        <v>0</v>
-      </c>
-      <c r="C143" s="15">
-        <v>0.060285605483625285</v>
-      </c>
-      <c r="D143" s="15">
-        <v>0.12028560548362528</v>
-      </c>
-      <c r="E143" s="15">
-        <v>0.03</v>
-      </c>
-      <c r="F143" s="15">
         <v>0.055</v>
       </c>
     </row>
@@ -5145,7 +3812,7 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="30" customWidth="1"/>
   </cols>
   <sheetData>
@@ -5191,7 +3858,7 @@
     </row>
     <row r="5" ht="36" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -5203,7 +3870,7 @@
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
@@ -5228,13 +3895,13 @@
     <row r="8" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="C9" s="6" t="s">
         <v>31</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -5245,7 +3912,7 @@
         <v>6.5</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -5256,7 +3923,7 @@
         <v>6.5</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -5267,7 +3934,7 @@
         <v>6.5</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -5278,7 +3945,7 @@
         <v>6.5</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -5289,7 +3956,7 @@
         <v>6.5</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -5300,7 +3967,7 @@
         <v>6.5</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -5311,7 +3978,7 @@
         <v>6.5</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -5329,11 +3996,11 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H128"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5378,7 +4045,7 @@
     </row>
     <row r="5" ht="36" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -5390,7 +4057,7 @@
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
@@ -5415,961 +4082,281 @@
     <row r="8" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="12">
-        <v>43739</v>
+        <v>46326</v>
       </c>
       <c r="B10" s="16">
-        <v>0.263</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="12">
-        <v>43770</v>
+        <v>46356</v>
       </c>
       <c r="B11" s="16">
-        <v>0</v>
+        <v>0.693</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="12">
-        <v>43800</v>
+        <v>46387</v>
       </c>
       <c r="B12" s="16">
-        <v>0.493</v>
+        <v>4.348</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="12">
-        <v>43831</v>
+        <v>46418</v>
       </c>
       <c r="B13" s="16">
-        <v>3.305</v>
+        <v>19.448</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="12">
-        <v>43862</v>
+        <v>46446</v>
       </c>
       <c r="B14" s="16">
-        <v>16.809</v>
+        <v>21.693</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="12">
-        <v>43891</v>
+        <v>46477</v>
       </c>
       <c r="B15" s="16">
-        <v>17.337</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="12">
-        <v>43922</v>
+        <v>46507</v>
       </c>
       <c r="B16" s="16">
-        <v>0</v>
+        <v>25.89</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="12">
-        <v>43952</v>
+        <v>46538</v>
       </c>
       <c r="B17" s="16">
-        <v>1.592</v>
+        <v>40.362</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="12">
-        <v>43983</v>
+        <v>46568</v>
       </c>
       <c r="B18" s="16">
-        <v>46.679</v>
+        <v>49.877</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="12">
-        <v>44013</v>
+        <v>46599</v>
       </c>
       <c r="B19" s="16">
-        <v>42.171</v>
+        <v>18.691</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="12">
-        <v>44044</v>
+        <v>46630</v>
       </c>
       <c r="B20" s="16">
-        <v>13.681</v>
+        <v>3.975</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="12">
-        <v>44075</v>
+        <v>46660</v>
       </c>
       <c r="B21" s="16">
-        <v>3.689</v>
+        <v>14.479</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="12">
-        <v>44105</v>
+        <v>46691</v>
       </c>
       <c r="B22" s="16">
-        <v>12.382</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="12">
-        <v>44136</v>
+        <v>46721</v>
       </c>
       <c r="B23" s="16">
-        <v>0</v>
+        <v>0.693</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="12">
-        <v>44166</v>
+        <v>46752</v>
       </c>
       <c r="B24" s="16">
-        <v>0.589</v>
+        <v>4.348</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="12">
-        <v>44197</v>
+        <v>46783</v>
       </c>
       <c r="B25" s="16">
-        <v>3.817</v>
+        <v>19.448</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="12">
-        <v>44228</v>
+        <v>46811</v>
       </c>
       <c r="B26" s="16">
-        <v>18.483</v>
+        <v>21.693</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="12">
-        <v>44256</v>
+        <v>46842</v>
       </c>
       <c r="B27" s="16">
-        <v>21.037</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="12">
-        <v>44287</v>
+        <v>46872</v>
       </c>
       <c r="B28" s="16">
-        <v>0</v>
+        <v>25.89</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="12">
-        <v>44317</v>
+        <v>46903</v>
       </c>
       <c r="B29" s="16">
-        <v>14.833</v>
+        <v>40.362</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="12">
-        <v>44348</v>
+        <v>46933</v>
       </c>
       <c r="B30" s="16">
-        <v>40.774</v>
+        <v>49.877</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="12">
-        <v>44378</v>
+        <v>46964</v>
       </c>
       <c r="B31" s="16">
-        <v>49.462</v>
+        <v>18.691</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="12">
-        <v>44409</v>
+        <v>46995</v>
       </c>
       <c r="B32" s="16">
-        <v>16.618</v>
+        <v>3.975</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="12">
-        <v>44440</v>
+        <v>47025</v>
       </c>
       <c r="B33" s="16">
-        <v>3.785</v>
+        <v>14.479</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="12">
-        <v>44470</v>
+        <v>47056</v>
       </c>
       <c r="B34" s="16">
-        <v>13.452</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="12">
-        <v>44501</v>
+        <v>47086</v>
       </c>
       <c r="B35" s="16">
-        <v>0</v>
+        <v>0.693</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="12">
-        <v>44531</v>
+        <v>47117</v>
       </c>
       <c r="B36" s="16">
-        <v>0.693</v>
+        <v>4.348</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="12">
-        <v>44562</v>
+        <v>47148</v>
       </c>
       <c r="B37" s="16">
-        <v>4.348</v>
+        <v>19.448</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="12">
-        <v>44593</v>
+        <v>47176</v>
       </c>
       <c r="B38" s="16">
-        <v>19.448</v>
+        <v>21.693</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="12">
-        <v>44621</v>
+        <v>47207</v>
       </c>
       <c r="B39" s="16">
-        <v>21.693</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="12">
-        <v>44652</v>
+        <v>47237</v>
       </c>
       <c r="B40" s="16">
-        <v>0</v>
+        <v>25.89</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="12">
-        <v>44682</v>
+        <v>47268</v>
       </c>
       <c r="B41" s="16">
-        <v>25.89</v>
+        <v>40.362</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="12">
-        <v>44713</v>
+        <v>47298</v>
       </c>
       <c r="B42" s="16">
-        <v>40.362</v>
+        <v>49.877</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="12">
-        <v>44743</v>
+        <v>47329</v>
       </c>
       <c r="B43" s="16">
-        <v>49.877</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A44" s="12">
-        <v>44774</v>
-      </c>
-      <c r="B44" s="16">
-        <v>18.691</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A45" s="12">
-        <v>44805</v>
-      </c>
-      <c r="B45" s="16">
-        <v>3.975</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A46" s="12">
-        <v>44835</v>
-      </c>
-      <c r="B46" s="16">
-        <v>14.479</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A47" s="12">
-        <v>44866</v>
-      </c>
-      <c r="B47" s="16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A48" s="12">
-        <v>44896</v>
-      </c>
-      <c r="B48" s="16">
-        <v>0.693</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A49" s="12">
-        <v>44927</v>
-      </c>
-      <c r="B49" s="16">
-        <v>4.348</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A50" s="12">
-        <v>44958</v>
-      </c>
-      <c r="B50" s="16">
-        <v>19.448</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A51" s="12">
-        <v>44986</v>
-      </c>
-      <c r="B51" s="16">
-        <v>21.693</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A52" s="12">
-        <v>45017</v>
-      </c>
-      <c r="B52" s="16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A53" s="12">
-        <v>45047</v>
-      </c>
-      <c r="B53" s="16">
-        <v>25.89</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A54" s="12">
-        <v>45078</v>
-      </c>
-      <c r="B54" s="16">
-        <v>40.362</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A55" s="12">
-        <v>45108</v>
-      </c>
-      <c r="B55" s="16">
-        <v>49.877</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A56" s="12">
-        <v>45139</v>
-      </c>
-      <c r="B56" s="16">
-        <v>18.691</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A57" s="12">
-        <v>45170</v>
-      </c>
-      <c r="B57" s="16">
-        <v>3.975</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A58" s="12">
-        <v>45200</v>
-      </c>
-      <c r="B58" s="16">
-        <v>14.479</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A59" s="12">
-        <v>45231</v>
-      </c>
-      <c r="B59" s="16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A60" s="12">
-        <v>45261</v>
-      </c>
-      <c r="B60" s="16">
-        <v>0.693</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A61" s="12">
-        <v>45292</v>
-      </c>
-      <c r="B61" s="16">
-        <v>4.348</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A62" s="12">
-        <v>45323</v>
-      </c>
-      <c r="B62" s="16">
-        <v>19.448</v>
-      </c>
-    </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A63" s="12">
-        <v>45351</v>
-      </c>
-      <c r="B63" s="16">
-        <v>21.693</v>
-      </c>
-    </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A64" s="12">
-        <v>45382</v>
-      </c>
-      <c r="B64" s="16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A65" s="12">
-        <v>45412</v>
-      </c>
-      <c r="B65" s="16">
-        <v>25.89</v>
-      </c>
-    </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A66" s="12">
-        <v>45443</v>
-      </c>
-      <c r="B66" s="16">
-        <v>40.362</v>
-      </c>
-    </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A67" s="12">
-        <v>45473</v>
-      </c>
-      <c r="B67" s="16">
-        <v>49.877</v>
-      </c>
-    </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A68" s="12">
-        <v>45504</v>
-      </c>
-      <c r="B68" s="16">
-        <v>18.691</v>
-      </c>
-    </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A69" s="12">
-        <v>45535</v>
-      </c>
-      <c r="B69" s="16">
-        <v>3.975</v>
-      </c>
-    </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A70" s="12">
-        <v>45565</v>
-      </c>
-      <c r="B70" s="16">
-        <v>14.479</v>
-      </c>
-    </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A71" s="12">
-        <v>45596</v>
-      </c>
-      <c r="B71" s="16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A72" s="12">
-        <v>45626</v>
-      </c>
-      <c r="B72" s="16">
-        <v>0.693</v>
-      </c>
-    </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A73" s="12">
-        <v>45657</v>
-      </c>
-      <c r="B73" s="16">
-        <v>4.348</v>
-      </c>
-    </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A74" s="12">
-        <v>45688</v>
-      </c>
-      <c r="B74" s="16">
-        <v>19.448</v>
-      </c>
-    </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A75" s="12">
-        <v>45716</v>
-      </c>
-      <c r="B75" s="16">
-        <v>21.693</v>
-      </c>
-    </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A76" s="12">
-        <v>45747</v>
-      </c>
-      <c r="B76" s="16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A77" s="12">
-        <v>45777</v>
-      </c>
-      <c r="B77" s="16">
-        <v>25.89</v>
-      </c>
-    </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A78" s="12">
-        <v>45808</v>
-      </c>
-      <c r="B78" s="16">
-        <v>40.362</v>
-      </c>
-    </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A79" s="12">
-        <v>45838</v>
-      </c>
-      <c r="B79" s="16">
-        <v>49.877</v>
-      </c>
-    </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A80" s="12">
-        <v>45869</v>
-      </c>
-      <c r="B80" s="16">
-        <v>18.691</v>
-      </c>
-    </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A81" s="12">
-        <v>45900</v>
-      </c>
-      <c r="B81" s="16">
-        <v>3.975</v>
-      </c>
-    </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A82" s="12">
-        <v>45930</v>
-      </c>
-      <c r="B82" s="16">
-        <v>14.479</v>
-      </c>
-    </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A83" s="12">
-        <v>45961</v>
-      </c>
-      <c r="B83" s="16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A84" s="12">
-        <v>45991</v>
-      </c>
-      <c r="B84" s="16">
-        <v>0.693</v>
-      </c>
-    </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A85" s="12">
-        <v>46022</v>
-      </c>
-      <c r="B85" s="16">
-        <v>4.348</v>
-      </c>
-    </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A86" s="12">
-        <v>46053</v>
-      </c>
-      <c r="B86" s="16">
-        <v>19.448</v>
-      </c>
-    </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A87" s="12">
-        <v>46081</v>
-      </c>
-      <c r="B87" s="16">
-        <v>21.693</v>
-      </c>
-    </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A88" s="12">
-        <v>46112</v>
-      </c>
-      <c r="B88" s="16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A89" s="12">
-        <v>46142</v>
-      </c>
-      <c r="B89" s="16">
-        <v>25.89</v>
-      </c>
-    </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A90" s="12">
-        <v>46173</v>
-      </c>
-      <c r="B90" s="16">
-        <v>40.362</v>
-      </c>
-    </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A91" s="12">
-        <v>46203</v>
-      </c>
-      <c r="B91" s="16">
-        <v>49.877</v>
-      </c>
-    </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A92" s="12">
-        <v>46234</v>
-      </c>
-      <c r="B92" s="16">
-        <v>18.691</v>
-      </c>
-    </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A93" s="12">
-        <v>46265</v>
-      </c>
-      <c r="B93" s="16">
-        <v>3.975</v>
-      </c>
-    </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A94" s="12">
-        <v>46295</v>
-      </c>
-      <c r="B94" s="16">
-        <v>14.479</v>
-      </c>
-    </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A95" s="12">
-        <v>46326</v>
-      </c>
-      <c r="B95" s="16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A96" s="12">
-        <v>46356</v>
-      </c>
-      <c r="B96" s="16">
-        <v>0.693</v>
-      </c>
-    </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A97" s="12">
-        <v>46387</v>
-      </c>
-      <c r="B97" s="16">
-        <v>4.348</v>
-      </c>
-    </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A98" s="12">
-        <v>46418</v>
-      </c>
-      <c r="B98" s="16">
-        <v>19.448</v>
-      </c>
-    </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A99" s="12">
-        <v>46446</v>
-      </c>
-      <c r="B99" s="16">
-        <v>21.693</v>
-      </c>
-    </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A100" s="12">
-        <v>46477</v>
-      </c>
-      <c r="B100" s="16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A101" s="12">
-        <v>46507</v>
-      </c>
-      <c r="B101" s="16">
-        <v>25.89</v>
-      </c>
-    </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A102" s="12">
-        <v>46538</v>
-      </c>
-      <c r="B102" s="16">
-        <v>40.362</v>
-      </c>
-    </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A103" s="12">
-        <v>46568</v>
-      </c>
-      <c r="B103" s="16">
-        <v>49.877</v>
-      </c>
-    </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A104" s="12">
-        <v>46599</v>
-      </c>
-      <c r="B104" s="16">
-        <v>18.691</v>
-      </c>
-    </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A105" s="12">
-        <v>46630</v>
-      </c>
-      <c r="B105" s="16">
-        <v>3.975</v>
-      </c>
-    </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A106" s="12">
-        <v>46660</v>
-      </c>
-      <c r="B106" s="16">
-        <v>14.479</v>
-      </c>
-    </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A107" s="12">
-        <v>46691</v>
-      </c>
-      <c r="B107" s="16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A108" s="12">
-        <v>46721</v>
-      </c>
-      <c r="B108" s="16">
-        <v>0.693</v>
-      </c>
-    </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A109" s="12">
-        <v>46752</v>
-      </c>
-      <c r="B109" s="16">
-        <v>4.348</v>
-      </c>
-    </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A110" s="12">
-        <v>46783</v>
-      </c>
-      <c r="B110" s="16">
-        <v>19.448</v>
-      </c>
-    </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A111" s="12">
-        <v>46811</v>
-      </c>
-      <c r="B111" s="16">
-        <v>21.693</v>
-      </c>
-    </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A112" s="12">
-        <v>46842</v>
-      </c>
-      <c r="B112" s="16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A113" s="12">
-        <v>46872</v>
-      </c>
-      <c r="B113" s="16">
-        <v>25.89</v>
-      </c>
-    </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A114" s="12">
-        <v>46903</v>
-      </c>
-      <c r="B114" s="16">
-        <v>40.362</v>
-      </c>
-    </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A115" s="12">
-        <v>46933</v>
-      </c>
-      <c r="B115" s="16">
-        <v>49.877</v>
-      </c>
-    </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A116" s="12">
-        <v>46964</v>
-      </c>
-      <c r="B116" s="16">
-        <v>18.691</v>
-      </c>
-    </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A117" s="12">
-        <v>46995</v>
-      </c>
-      <c r="B117" s="16">
-        <v>3.975</v>
-      </c>
-    </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A118" s="12">
-        <v>47025</v>
-      </c>
-      <c r="B118" s="16">
-        <v>14.479</v>
-      </c>
-    </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A119" s="12">
-        <v>47056</v>
-      </c>
-      <c r="B119" s="16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A120" s="12">
-        <v>47086</v>
-      </c>
-      <c r="B120" s="16">
-        <v>0.693</v>
-      </c>
-    </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A121" s="12">
-        <v>47117</v>
-      </c>
-      <c r="B121" s="16">
-        <v>4.348</v>
-      </c>
-    </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A122" s="12">
-        <v>47148</v>
-      </c>
-      <c r="B122" s="16">
-        <v>19.448</v>
-      </c>
-    </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A123" s="12">
-        <v>47176</v>
-      </c>
-      <c r="B123" s="16">
-        <v>21.693</v>
-      </c>
-    </row>
-    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A124" s="12">
-        <v>47207</v>
-      </c>
-      <c r="B124" s="16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A125" s="12">
-        <v>47237</v>
-      </c>
-      <c r="B125" s="16">
-        <v>25.89</v>
-      </c>
-    </row>
-    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A126" s="12">
-        <v>47268</v>
-      </c>
-      <c r="B126" s="16">
-        <v>40.362</v>
-      </c>
-    </row>
-    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A127" s="12">
-        <v>47298</v>
-      </c>
-      <c r="B127" s="16">
-        <v>49.877</v>
-      </c>
-    </row>
-    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A128" s="12">
-        <v>47329</v>
-      </c>
-      <c r="B128" s="16">
         <v>18.691</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Round 10: workbook mapping, golden tests, crawls, per strike type and side, white surfaces, sign-off prep
Mapping doc and verify:mapping for every workbook formula cell; G0 compares 4,497 saved values; G1 to G6 and fast-check invariants; stage spy test; API contracts for every route; number, button, layout and pipeline crawls; strike matrix; no-protection products; loss-cap warning; stale runs hidden from the Atlas and Excel; lib/excel and lib/underlyings; Linux only visual baselines; docs 11 to 13.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/samples/Hedging_Sheet_Vol_Surface_Sample.xlsx
+++ b/public/samples/Hedging_Sheet_Vol_Surface_Sample.xlsx
@@ -1252,7 +1252,7 @@
         <v>46203</v>
       </c>
       <c r="B13" s="13">
-        <v>50.9</v>
+        <v>53.5</v>
       </c>
       <c r="C13" s="13">
         <v>53.5</v>
@@ -1320,7 +1320,7 @@
         <v>46231</v>
       </c>
       <c r="B14" s="13">
-        <v>50.9</v>
+        <v>46.24</v>
       </c>
       <c r="C14" s="13">
         <v>46.24</v>
@@ -1388,7 +1388,7 @@
         <v>46259</v>
       </c>
       <c r="B15" s="13">
-        <v>45.12</v>
+        <v>46.12</v>
       </c>
       <c r="C15" s="13">
         <v>46.12</v>
@@ -1456,7 +1456,7 @@
         <v>46294</v>
       </c>
       <c r="B16" s="13">
-        <v>41.94</v>
+        <v>38.38</v>
       </c>
       <c r="C16" s="13">
         <v>38.38</v>
@@ -1524,7 +1524,7 @@
         <v>46322</v>
       </c>
       <c r="B17" s="13">
-        <v>35.68</v>
+        <v>37.26</v>
       </c>
       <c r="C17" s="13">
         <v>37.26</v>
@@ -1592,7 +1592,7 @@
         <v>46385</v>
       </c>
       <c r="B18" s="13">
-        <v>35.68</v>
+        <v>33.39</v>
       </c>
       <c r="C18" s="13">
         <v>33.39</v>
@@ -1660,7 +1660,7 @@
         <v>46476</v>
       </c>
       <c r="B19" s="13">
-        <v>31.5</v>
+        <v>30.78</v>
       </c>
       <c r="C19" s="13">
         <v>30.78</v>
@@ -1728,7 +1728,7 @@
         <v>46567</v>
       </c>
       <c r="B20" s="13">
-        <v>29.84</v>
+        <v>28.9</v>
       </c>
       <c r="C20" s="13">
         <v>28.9</v>
@@ -1796,7 +1796,7 @@
         <v>46658</v>
       </c>
       <c r="B21" s="13">
-        <v>28.45</v>
+        <v>28.22</v>
       </c>
       <c r="C21" s="13">
         <v>28.22</v>
@@ -1864,7 +1864,7 @@
         <v>46749</v>
       </c>
       <c r="B22" s="13">
-        <v>27.36</v>
+        <v>27.57</v>
       </c>
       <c r="C22" s="13">
         <v>27.57</v>
@@ -1932,7 +1932,7 @@
         <v>46840</v>
       </c>
       <c r="B23" s="13">
-        <v>26.78</v>
+        <v>26.95</v>
       </c>
       <c r="C23" s="13">
         <v>26.95</v>
@@ -2000,7 +2000,7 @@
         <v>46931</v>
       </c>
       <c r="B24" s="13">
-        <v>26.16</v>
+        <v>26.49</v>
       </c>
       <c r="C24" s="13">
         <v>26.49</v>
@@ -2068,7 +2068,7 @@
         <v>47113</v>
       </c>
       <c r="B25" s="13">
-        <v>25.55</v>
+        <v>26.02</v>
       </c>
       <c r="C25" s="13">
         <v>26.02</v>
@@ -2136,7 +2136,7 @@
         <v>47295</v>
       </c>
       <c r="B26" s="13">
-        <v>25.1</v>
+        <v>25.71</v>
       </c>
       <c r="C26" s="13">
         <v>25.71</v>
@@ -2204,7 +2204,7 @@
         <v>47476</v>
       </c>
       <c r="B27" s="13">
-        <v>24.52</v>
+        <v>25.74</v>
       </c>
       <c r="C27" s="13">
         <v>25.74</v>
@@ -2272,7 +2272,7 @@
         <v>47846</v>
       </c>
       <c r="B28" s="13">
-        <v>28.46</v>
+        <v>25.74</v>
       </c>
       <c r="C28" s="13">
         <v>25.74</v>
@@ -2340,7 +2340,7 @@
         <v>47878</v>
       </c>
       <c r="B29" s="13">
-        <v>28.46</v>
+        <v>25.74</v>
       </c>
       <c r="C29" s="13">
         <v>25.74</v>
@@ -2408,7 +2408,7 @@
         <v>47962</v>
       </c>
       <c r="B30" s="13">
-        <v>28.46</v>
+        <v>25.74</v>
       </c>
       <c r="C30" s="13">
         <v>25.74</v>

</xml_diff>